<commit_message>
Fill register with 10 sample rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011P5seQxeXE2hwCFZfyN971
</commit_message>
<xml_diff>
--- a/18 октября/Реестр решений и деклараций.xlsx
+++ b/18 октября/Реестр решений и деклараций.xlsx
@@ -498,151 +498,331 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="80" customHeight="1">
       <c r="A2" s="2">
         <f>IF(B2="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0145/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: отбор проб, определение состава</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>50508/020926/0011452</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Выпуск разрешён, код ТН ВЭД подтверждён</t>
+        </is>
+      </c>
       <c r="G2" s="2">
         <f>IF(B2="","","Решение № "&amp;B2&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C2&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D2="","",TEXT(DAY(D2),"00")&amp;"."&amp;TEXT(MONTH(D2),"00")&amp;"."&amp;YEAR(D2))&amp;CHAR(10)&amp;"Декларация № "&amp;E2&amp;CHAR(10)&amp;"Комментарий: "&amp;F2)</f>
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="80" customHeight="1">
       <c r="A3" s="2">
         <f>IF(B3="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0152/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: идентификация товара</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46270</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>50508/050926/0011687</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Выпуск под обеспечение, ожидается заключение ЦТЛ</t>
+        </is>
+      </c>
       <c r="G3" s="2">
         <f>IF(B3="","","Решение № "&amp;B3&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C3&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D3="","",TEXT(DAY(D3),"00")&amp;"."&amp;TEXT(MONTH(D3),"00")&amp;"."&amp;YEAR(D3))&amp;CHAR(10)&amp;"Декларация № "&amp;E3&amp;CHAR(10)&amp;"Комментарий: "&amp;F3)</f>
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="2">
         <f>IF(B4="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0163/2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: определение страны происхождения</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>50508/090926/0012034</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Заключение получено, корректировка не требуется</t>
+        </is>
+      </c>
       <c r="G4" s="2">
         <f>IF(B4="","","Решение № "&amp;B4&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C4&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D4="","",TEXT(DAY(D4),"00")&amp;"."&amp;TEXT(MONTH(D4),"00")&amp;"."&amp;YEAR(D4))&amp;CHAR(10)&amp;"Декларация № "&amp;E4&amp;CHAR(10)&amp;"Комментарий: "&amp;F4)</f>
         <v/>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="80" customHeight="1">
       <c r="A5" s="2">
         <f>IF(B5="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0171/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: химический анализ</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>50508/120926/0012311</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Код ТН ВЭД изменён, доначислены платежи</t>
+        </is>
+      </c>
       <c r="G5" s="2">
         <f>IF(B5="","","Решение № "&amp;B5&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C5&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D5="","",TEXT(DAY(D5),"00")&amp;"."&amp;TEXT(MONTH(D5),"00")&amp;"."&amp;YEAR(D5))&amp;CHAR(10)&amp;"Декларация № "&amp;E5&amp;CHAR(10)&amp;"Комментарий: "&amp;F5)</f>
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="2">
         <f>IF(B6="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0184/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: экспертиза маркировки</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>50508/170926/0012795</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Выпуск разрешён, замечаний нет</t>
+        </is>
+      </c>
       <c r="G6" s="2">
         <f>IF(B6="","","Решение № "&amp;B6&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C6&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D6="","",TEXT(DAY(D6),"00")&amp;"."&amp;TEXT(MONTH(D6),"00")&amp;"."&amp;YEAR(D6))&amp;CHAR(10)&amp;"Декларация № "&amp;E6&amp;CHAR(10)&amp;"Комментарий: "&amp;F6)</f>
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2">
         <f>IF(B7="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0196/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: определение таможенной стоимости</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>50508/220926/0013148</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Запрошены доп. документы у декларанта</t>
+        </is>
+      </c>
       <c r="G7" s="2">
         <f>IF(B7="","","Решение № "&amp;B7&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C7&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D7="","",TEXT(DAY(D7),"00")&amp;"."&amp;TEXT(MONTH(D7),"00")&amp;"."&amp;YEAR(D7))&amp;CHAR(10)&amp;"Декларация № "&amp;E7&amp;CHAR(10)&amp;"Комментарий: "&amp;F7)</f>
         <v/>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2">
         <f>IF(B8="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0203/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: отбор проб, анализ состава</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>50508/260926/0013502</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Подана КДТ, ожидается решение</t>
+        </is>
+      </c>
       <c r="G8" s="2">
         <f>IF(B8="","","Решение № "&amp;B8&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C8&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D8="","",TEXT(DAY(D8),"00")&amp;"."&amp;TEXT(MONTH(D8),"00")&amp;"."&amp;YEAR(D8))&amp;CHAR(10)&amp;"Декларация № "&amp;E8&amp;CHAR(10)&amp;"Комментарий: "&amp;F8)</f>
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2">
         <f>IF(B9="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0215/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: идентификация оборудования</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>50508/011026/0013960</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Выпуск разрешён, образцы возвращены</t>
+        </is>
+      </c>
       <c r="G9" s="2">
         <f>IF(B9="","","Решение № "&amp;B9&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C9&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D9="","",TEXT(DAY(D9),"00")&amp;"."&amp;TEXT(MONTH(D9),"00")&amp;"."&amp;YEAR(D9))&amp;CHAR(10)&amp;"Декларация № "&amp;E9&amp;CHAR(10)&amp;"Комментарий: "&amp;F9)</f>
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2">
         <f>IF(B10="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0228/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: товароведческая экспертиза</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>50508/071026/0014417</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Заключение ЦТЛ на рассмотрении</t>
+        </is>
+      </c>
       <c r="G10" s="2">
         <f>IF(B10="","","Решение № "&amp;B10&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C10&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D10="","",TEXT(DAY(D10),"00")&amp;"."&amp;TEXT(MONTH(D10),"00")&amp;"."&amp;YEAR(D10))&amp;CHAR(10)&amp;"Декларация № "&amp;E10&amp;CHAR(10)&amp;"Комментарий: "&amp;F10)</f>
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2">
         <f>IF(B11="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>РШ-0236/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Направлено: определение состава текстиля</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>50508/141026/0014873</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Выпуск разрешён, обеспечение возвращено</t>
+        </is>
+      </c>
       <c r="G11" s="2">
         <f>IF(B11="","","Решение № "&amp;B11&amp;CHAR(10)&amp;"Направление в ЦТЛ: "&amp;C11&amp;CHAR(10)&amp;"Дата решения: "&amp;IF(D11="","",TEXT(DAY(D11),"00")&amp;"."&amp;TEXT(MONTH(D11),"00")&amp;"."&amp;YEAR(D11))&amp;CHAR(10)&amp;"Декларация № "&amp;E11&amp;CHAR(10)&amp;"Комментарий: "&amp;F11)</f>
         <v/>

</xml_diff>

<commit_message>
Keep only the summary column in register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011P5seQxeXE2hwCFZfyN971
</commit_message>
<xml_diff>
--- a/18 октября/Реестр решений и деклараций.xlsx
+++ b/18 октября/Реестр решений и деклараций.xlsx
@@ -7,20 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр'!$A$1:$G$11</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -73,15 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -449,83 +442,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Номер решения</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Направление в ЦТЛ</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Дата решения</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Номер декларации</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Комментарий после выпуска декларации</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Сводка (всё в одной ячейке)</t>
+          <t>Сводка</t>
         </is>
       </c>
     </row>
     <row r="2" ht="80" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0145/2026</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: отбор проб, определение состава</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>46267</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>50508/020926/0011452</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Выпуск разрешён, код ТН ВЭД подтверждён</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0145/2026
 Направление в ЦТЛ: Направлено: отбор проб, определение состава
@@ -536,33 +467,7 @@
       </c>
     </row>
     <row r="3" ht="80" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0152/2026</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: идентификация товара</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>46270</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>50508/050926/0011687</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Выпуск под обеспечение, ожидается заключение ЦТЛ</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0152/2026
 Направление в ЦТЛ: Направлено: идентификация товара
@@ -573,33 +478,7 @@
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0163/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: определение страны происхождения</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>46274</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>50508/090926/0012034</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Заключение получено, корректировка не требуется</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0163/2026
 Направление в ЦТЛ: Направлено: определение страны происхождения
@@ -610,33 +489,7 @@
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0171/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: химический анализ</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>50508/120926/0012311</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Код ТН ВЭД изменён, доначислены платежи</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0171/2026
 Направление в ЦТЛ: Направлено: химический анализ
@@ -647,33 +500,7 @@
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0184/2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: экспертиза маркировки</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>46282</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>50508/170926/0012795</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Выпуск разрешён, замечаний нет</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0184/2026
 Направление в ЦТЛ: Направлено: экспертиза маркировки
@@ -684,33 +511,7 @@
       </c>
     </row>
     <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0196/2026</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: определение таможенной стоимости</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>46287</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>50508/220926/0013148</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Запрошены доп. документы у декларанта</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0196/2026
 Направление в ЦТЛ: Направлено: определение таможенной стоимости
@@ -721,33 +522,7 @@
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0203/2026</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: отбор проб, анализ состава</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>46291</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>50508/260926/0013502</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Подана КДТ, ожидается решение</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0203/2026
 Направление в ЦТЛ: Направлено: отбор проб, анализ состава
@@ -758,33 +533,7 @@
       </c>
     </row>
     <row r="9" ht="80" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0215/2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: идентификация оборудования</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>50508/011026/0013960</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Выпуск разрешён, образцы возвращены</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0215/2026
 Направление в ЦТЛ: Направлено: идентификация оборудования
@@ -795,33 +544,7 @@
       </c>
     </row>
     <row r="10" ht="80" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0228/2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: товароведческая экспертиза</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>46302</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>50508/071026/0014417</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Заключение ЦТЛ на рассмотрении</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0228/2026
 Направление в ЦТЛ: Направлено: товароведческая экспертиза
@@ -832,33 +555,7 @@
       </c>
     </row>
     <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>РШ-0236/2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Направлено: определение состава текстиля</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>50508/141026/0014873</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Выпуск разрешён, обеспечение возвращено</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Решение № РШ-0236/2026
 Направление в ЦТЛ: Направлено: определение состава текстиля
@@ -869,12 +566,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Введите дату" type="date" operator="greaterThan">
-      <formula1>DATE(2000,1,1)</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make register summary cells unstructured
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011P5seQxeXE2hwCFZfyN971
</commit_message>
<xml_diff>
--- a/18 октября/Реестр решений и деклараций.xlsx
+++ b/18 октября/Реестр решений и деклараций.xlsx
@@ -455,113 +455,82 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="80" customHeight="1">
+    <row r="2" ht="50" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0145/2026
-Направление в ЦТЛ: Направлено: отбор проб, определение состава
-Дата решения: 02.09.2026
-Декларация № 50508/020926/0011452
-Комментарий: Выпуск разрешён, код ТН ВЭД подтверждён</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="80" customHeight="1">
+          <t>ДТ 50508/020926/0011452 выпуск разрешён, код ТН ВЭД подтвердили; реш. РШ-0145/2026 от 02.09.26 — в ЦТЛ на отбор проб (состав)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0152/2026
-Направление в ЦТЛ: Направлено: идентификация товара
-Дата решения: 05.09.2026
-Декларация № 50508/050926/0011687
-Комментарий: Выпуск под обеспечение, ожидается заключение ЦТЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
+          <t>05/09/2026
+идентификация товара (ЦТЛ)
+выпущено под обеспечение, ждём заключение
+№ решения 0152/2026
+декл. 50508/050926/0011687</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0163/2026
-Направление в ЦТЛ: Направлено: определение страны происхождения
-Дата решения: 09.09.2026
-Декларация № 50508/090926/0012034
-Комментарий: Заключение получено, корректировка не требуется</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
+          <t>Комментарий: заключение пришло, корректировка не нужна. 50508/090926/0012034. Решение РШ-0163/2026, 9 сентября 2026, ЦТЛ - страна происхождения</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0171/2026
-Направление в ЦТЛ: Направлено: химический анализ
-Дата решения: 12.09.2026
-Декларация № 50508/120926/0012311
-Комментарий: Код ТН ВЭД изменён, доначислены платежи</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
+          <t>РШ-0171/2026 хим. анализ 12.09.2026 ДТ: 50508/120926/0012311 код изменён!! доначислили платежи</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0184/2026
-Направление в ЦТЛ: Направлено: экспертиза маркировки
-Дата решения: 17.09.2026
-Декларация № 50508/170926/0012795
-Комментарий: Выпуск разрешён, замечаний нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
+          <t>маркировка → ЦТЛ / 17.09.26 / 50508/170926/0012795 / замечаний нет, выпуск ок / реш РШ-184</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0196/2026
-Направление в ЦТЛ: Направлено: определение таможенной стоимости
-Дата решения: 22.09.2026
-Декларация № 50508/220926/0013148
-Комментарий: Запрошены доп. документы у декларанта</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1">
+          <t>декларация 50508/220926/0013148
+запросили доп. документы у декларанта
+РШ-0196/2026
+ЦТЛ: тамож. стоимость
+22.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0203/2026
-Направление в ЦТЛ: Направлено: отбор проб, анализ состава
-Дата решения: 26.09.2026
-Декларация № 50508/260926/0013502
-Комментарий: Подана КДТ, ожидается решение</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="80" customHeight="1">
+          <t>26 сент. — отбор проб, анализ состава; КДТ подана, ждём решения; ДТ 50508/260926/0013502; решение № РШ-0203/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0215/2026
-Направление в ЦТЛ: Направлено: идентификация оборудования
-Дата решения: 01.10.2026
-Декларация № 50508/011026/0013960
-Комментарий: Выпуск разрешён, образцы возвращены</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="80" customHeight="1">
+          <t>Выпуск разрешён, образцы вернули. 1.10.2026 реш. РШ-0215/2026 (идентификация оборудования в ЦТЛ) ДТ 50508/011026/0013960</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0228/2026
-Направление в ЦТЛ: Направлено: товароведческая экспертиза
-Дата решения: 07.10.2026
-Декларация № 50508/071026/0014417
-Комментарий: Заключение ЦТЛ на рассмотрении</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="80" customHeight="1">
+          <t>50508/071026/0014417 — заключение ЦТЛ пока на рассмотрении
+товароведческая экспертиза, РШ-0228/2026, 07-10-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Решение № РШ-0236/2026
-Направление в ЦТЛ: Направлено: определение состава текстиля
-Дата решения: 14.10.2026
-Декларация № 50508/141026/0014873
-Комментарий: Выпуск разрешён, обеспечение возвращено</t>
+          <t>обеспечение вернули, выпуск разрешён;; ЦТЛ состав текстиля;; 14.10.26;; РШ 0236/2026;; ДТ№50508/141026/0014873</t>
         </is>
       </c>
     </row>

</xml_diff>